<commit_message>
fixed p values and graphs
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/Assignment-4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C94737E2-B8A0-4E53-B7CB-CFBC304837E3}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A3BC576-74A7-4355-9173-3D4F0D649FF7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -504,7 +504,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="4">
-        <v>-0.49031000000000002</v>
+        <v>0.25457999999999997</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -512,7 +512,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="4">
-        <v>-0.50117999999999996</v>
+        <v>2.0787</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -520,7 +520,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>-0.50156999999999996</v>
+        <v>2.9998999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -546,8 +546,9 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
local truncation error table
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/Assignment-4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A3BC576-74A7-4355-9173-3D4F0D649FF7}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="11_F25DC773A252ABDACC10482CB99841445ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2694E2D-7F72-4BAE-9D50-3047CF44D174}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Global Truncation Error Scaling vs. Step Size Table (Runge-Kutta)</t>
   </si>
@@ -43,6 +44,18 @@
   </si>
   <si>
     <t>Runga Kutta</t>
+  </si>
+  <si>
+    <t>Local Truncation Error Scaling Table, embedded RK</t>
+  </si>
+  <si>
+    <t>Higher Order</t>
+  </si>
+  <si>
+    <t>Lower Order</t>
+  </si>
+  <si>
+    <t>Difference |XB1-XB2|</t>
   </si>
 </sst>
 </file>
@@ -115,7 +128,82 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <family val="3"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -204,12 +292,27 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2155F23-4F3E-4171-9AA1-9C135615524A}" name="Table2" displayName="Table2" ref="A2:B5" totalsRowShown="0" headerRowDxfId="3" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2155F23-4F3E-4171-9AA1-9C135615524A}" name="Table2" displayName="Table2" ref="A2:B5" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A2:B5" xr:uid="{C2155F23-4F3E-4171-9AA1-9C135615524A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B6D33823-484C-480B-BD2B-50DAD0B26EEC}" name="Method" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{2BB2C435-8B64-4474-85CF-CFBA46640A6D}" name="p (-)" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{B6D33823-484C-480B-BD2B-50DAD0B26EEC}" name="Method" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{2BB2C435-8B64-4474-85CF-CFBA46640A6D}" name="p (-)" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B5786823-E529-48E4-9936-86B96BFF1B06}" name="Table22" displayName="Table22" ref="A2:B5" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+  <autoFilter ref="A2:B5" xr:uid="{B5786823-E529-48E4-9936-86B96BFF1B06}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{9BE7A584-E19B-4660-B782-B406D8988DF0}" name="Method" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{FFA84BD2-5BC6-45A2-A1E1-40A7F3CF7C1C}" name="p (-)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -551,4 +654,62 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DD88630-84F2-4216-A051-188E87090254}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="5"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2.9371999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2.8769</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1.0855999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>